<commit_message>
Revise 21 Sep minutes with Zhang Junfeng's roster and refresh the tracker
Replace informal names with the commander pre-meeting assignments, keep the original minutes outline, and ship Word plus PDF instead of a new markdown recap.

Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/meetings/POA生物制品项目改造-行动项跟踪.xlsx
+++ b/meetings/POA生物制品项目改造-行动项跟踪.xlsx
@@ -160,12 +160,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FADBD8"/>
+        <fgColor rgb="00D6EAF8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6EAF8"/>
+        <fgColor rgb="00FADBD8"/>
       </patternFill>
     </fill>
   </fills>
@@ -344,7 +344,7 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -597,62 +597,27 @@
   <commentList>
     <comment ref="E5" authorId="0" shapeId="0">
       <text>
-        <t>厂名转写或作东福龙 / 多福龙，按东富龙，待核实。</t>
-      </text>
-    </comment>
-    <comment ref="E10" authorId="0" shapeId="0">
-      <text>
-        <t>责任人全名待补。</t>
-      </text>
-    </comment>
-    <comment ref="E11" authorId="0" shapeId="0">
-      <text>
-        <t>亚光转写或作雅光，待核实。</t>
+        <t>人员以张俊峰会前消息为准。</t>
       </text>
     </comment>
     <comment ref="E12" authorId="0" shapeId="0">
       <text>
-        <t>对接人待补。</t>
-      </text>
-    </comment>
-    <comment ref="E14" authorId="0" shapeId="0">
-      <text>
-        <t>截止日期待方案列出后指定。</t>
+        <t>会前消息未点名汉邦，保留转写。</t>
       </text>
     </comment>
     <comment ref="E15" authorId="0" shapeId="0">
       <text>
-        <t>单一责任人按宋金柱；配合人见进展。</t>
+        <t>项目号 139788。</t>
+      </text>
+    </comment>
+    <comment ref="E16" authorId="0" shapeId="0">
+      <text>
+        <t>配合人：田子才。</t>
       </text>
     </comment>
     <comment ref="E17" authorId="0" shapeId="0">
       <text>
-        <t>门口搬运：泽鹏。拆卸转移：宋金柱。术语按项目指定：三合一 = AFD。</t>
-      </text>
-    </comment>
-    <comment ref="E19" authorId="0" shapeId="0">
-      <text>
-        <t>会上先说 C 区、后更正为 D 区现有罐改口，不是新建。位号待补。</t>
-      </text>
-    </comment>
-    <comment ref="E20" authorId="0" shapeId="0">
-      <text>
-        <t>与 A-20260921-11 联动：11 出架子，16 补新项。</t>
-      </text>
-    </comment>
-    <comment ref="E21" authorId="0" shapeId="0">
-      <text>
-        <t>截止日期按首场；此后每日重复。</t>
-      </text>
-    </comment>
-    <comment ref="E22" authorId="0" shapeId="0">
-      <text>
-        <t>截止日期会上未指定。</t>
-      </text>
-    </comment>
-    <comment ref="E23" authorId="0" shapeId="0">
-      <text>
-        <t>截止日期 10/20 为纪要推断，待核实。责任人待落到人名。</t>
+        <t>三合一 = AFD。</t>
       </text>
     </comment>
   </commentList>
@@ -1339,7 +1304,7 @@
     <row r="28">
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>最近会议：2026-09-21 部署会 09:03–09:29。纪要：meetings/2026/2026-09-21-poa-deployment.md。项目代码书面 POA、口述 KOA，待核实。</t>
+          <t>最近会议：2026-09-21 部署会。人员以张俊峰会前分工为准。纪要 Word：meetings/2026/2026-09-21-BLA改造沟通会会议纪要-修订.docx。项目 139788。</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1523,7 @@
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D5" s="30" t="inlineStr">
@@ -1568,17 +1533,17 @@
       </c>
       <c r="E5" s="29" t="inlineStr">
         <is>
-          <t>牵头东富龙现场，按设备本体 / 管道 / 仪表 / 阀门 / 泵查漏补缺，更新制备配液与超滤改造须知。</t>
+          <t>打印改造事项清单；与东富龙技术员逐管路、逐设备过制备配液和超滤，缺项补进同一清单。</t>
         </is>
       </c>
       <c r="F5" s="29" t="inlineStr">
         <is>
-          <t>缺项已写入表，可提交合并会。</t>
+          <t>清单已查漏补缺，可与下午沉淀对表合并。</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr">
         <is>
-          <t>志恒</t>
+          <t>王志恒</t>
         </is>
       </c>
       <c r="H5" s="28" t="n">
@@ -1596,7 +1561,7 @@
       </c>
       <c r="K5" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置。上午对接东富龙，作为 IP 设计总牵头，配合两名管理人员细化。</t>
+          <t>2026-09-21：总指挥会前指定。皮轶杰跟制备，张冬跟超滤，郭泽鹏随队。</t>
         </is>
       </c>
       <c r="L5" s="28" t="n">
@@ -1623,7 +1588,7 @@
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D6" s="30" t="inlineStr">
@@ -1633,17 +1598,17 @@
       </c>
       <c r="E6" s="29" t="inlineStr">
         <is>
-          <t>对接东富龙现场人员，完成上午车间勘察。</t>
+          <t>负责制备配液和制备工序整改；今日跟王志恒、东富龙走现场并跟踪本片段。</t>
         </is>
       </c>
       <c r="F6" s="29" t="inlineStr">
         <is>
-          <t>厂家到场并走完相关管路。</t>
+          <t>本片段事项有人跟，缺项已记入王志恒清单。</t>
         </is>
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
-          <t>李主任</t>
+          <t>皮轶杰</t>
         </is>
       </c>
       <c r="H6" s="28" t="n">
@@ -1661,7 +1626,7 @@
       </c>
       <c r="K6" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置，上午完成。</t>
+          <t>2026-09-21：总指挥会前指定。不是「李主任」对接厂家。</t>
         </is>
       </c>
       <c r="L6" s="28" t="n">
@@ -1688,7 +1653,7 @@
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D7" s="30" t="inlineStr">
@@ -1698,17 +1663,17 @@
       </c>
       <c r="E7" s="29" t="inlineStr">
         <is>
-          <t>跟点超滤片断现场勘察并记录缺项。</t>
+          <t>负责超滤工序整改；今日跟王志恒、东富龙走现场并记录缺项。</t>
         </is>
       </c>
       <c r="F7" s="29" t="inlineStr">
         <is>
-          <t>超滤缺项已记入改造须知表。</t>
+          <t>超滤缺项已记入同一清单。</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>张东</t>
+          <t>张冬</t>
         </is>
       </c>
       <c r="H7" s="28" t="n">
@@ -1726,7 +1691,7 @@
       </c>
       <c r="K7" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置。张东超滤设备接触少，现场以跟点记录为主。</t>
+          <t>2026-09-21：总指挥会前指定。姓名为张冬，不是张东。</t>
         </is>
       </c>
       <c r="L7" s="28" t="n">
@@ -1753,27 +1718,27 @@
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D8" s="30" t="inlineStr">
         <is>
-          <t>设计方案</t>
+          <t>沉淀</t>
         </is>
       </c>
       <c r="E8" s="29" t="inlineStr">
         <is>
-          <t>厂家技术配合结束后，梳理超滤 / 制备配液改造事项并提交下午会。</t>
+          <t>负责沉淀工序整改；13:00 跟王志恒、亚光过沉淀区域。</t>
         </is>
       </c>
       <c r="F8" s="29" t="inlineStr">
         <is>
-          <t>有可过会的梳理稿。</t>
+          <t>沉淀缺项已记入同一清单。</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr">
         <is>
-          <t>志鹏</t>
+          <t>韩瑞衡</t>
         </is>
       </c>
       <c r="H8" s="28" t="n">
@@ -1791,7 +1756,7 @@
       </c>
       <c r="K8" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置。电子 / 智能技术员与张东配合其现场工作。</t>
+          <t>2026-09-21：总指挥会前指定。姓名为韩瑞衡。</t>
         </is>
       </c>
       <c r="L8" s="28" t="n">
@@ -1818,7 +1783,7 @@
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D9" s="30" t="inlineStr">
@@ -1828,17 +1793,17 @@
       </c>
       <c r="E9" s="29" t="inlineStr">
         <is>
-          <t>按沉淀 / 超滤 / 制备三片断，评估客户访问问题是否举一反三全覆盖，写入表单。</t>
+          <t>梳理客户来访全部问题，核三个片段涉及整改的内容是否都举一反三、都有整改要求。</t>
         </is>
       </c>
       <c r="F9" s="29" t="inlineStr">
         <is>
-          <t>表单能看出跨片断覆盖与缺口。</t>
+          <t>三个片段的覆盖与缺口写得清楚。</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
         <is>
-          <t>松涛</t>
+          <t>范兴涛</t>
         </is>
       </c>
       <c r="H9" s="28" t="n">
@@ -1856,7 +1821,7 @@
       </c>
       <c r="K9" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置。避免只改被点名的片断。</t>
+          <t>2026-09-21：总指挥会前指定。不是「松涛」。</t>
         </is>
       </c>
       <c r="L9" s="28" t="n">
@@ -1883,7 +1848,7 @@
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>王（IAP）</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D10" s="30" t="inlineStr">
@@ -1893,17 +1858,17 @@
       </c>
       <c r="E10" s="29" t="inlineStr">
         <is>
-          <t>通知东富龙曹工 / 赵工上午到场勘察利旧，下午交出利旧与推倒两套方案对比。</t>
+          <t>对接东富龙，下午交出利旧与推倒重建两套方案的时间/事项对比。</t>
         </is>
       </c>
       <c r="F10" s="29" t="inlineStr">
         <is>
-          <t>两套方案的事项与时间可对比。</t>
+          <t>两套方案可对比。</t>
         </is>
       </c>
       <c r="G10" s="27" t="inlineStr">
         <is>
-          <t>王（IAP，全名待补）</t>
+          <t>王志恒</t>
         </is>
       </c>
       <c r="H10" s="28" t="n">
@@ -1921,7 +1886,7 @@
       </c>
       <c r="K10" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：会上要求马上打电话；群里已催。下午与内部清单一起看。</t>
+          <t>2026-09-21：会上要求厂家出两套方案。</t>
         </is>
       </c>
       <c r="L10" s="28" t="n">
@@ -1948,27 +1913,27 @@
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>
-          <t>设计方案</t>
+          <t>沉淀</t>
         </is>
       </c>
       <c r="E11" s="29" t="inlineStr">
         <is>
-          <t>13:00 与亚光（菊工）合并昨天下午勘察事项与内部清单。</t>
+          <t>13:00 与亚光技术员梳理沉淀区域整改项，更新同一份改造清单。</t>
         </is>
       </c>
       <c r="F11" s="29" t="inlineStr">
         <is>
-          <t>合并清单一版。</t>
+          <t>沉淀项已并入清单。</t>
         </is>
       </c>
       <c r="G11" s="27" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>王志恒</t>
         </is>
       </c>
       <c r="H11" s="28" t="n">
@@ -1986,7 +1951,7 @@
       </c>
       <c r="K11" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置。昨日已把陈店 / 沉淀相关区域设备管道勘察一遍。</t>
+          <t>2026-09-21：总指挥会前指定。不是全员内部会。韩瑞衡现场跟。</t>
         </is>
       </c>
       <c r="L11" s="28" t="n">
@@ -2013,7 +1978,7 @@
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D12" s="30" t="inlineStr">
@@ -2033,7 +1998,7 @@
       </c>
       <c r="G12" s="27" t="inlineStr">
         <is>
-          <t>汉邦对接人（待补）</t>
+          <t>王志恒</t>
         </is>
       </c>
       <c r="H12" s="28" t="n">
@@ -2046,12 +2011,12 @@
       </c>
       <c r="J12" s="30" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="K12" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置，下午到场。</t>
+          <t>2026-09-21：转写提到下午汉邦到场。对接人若另有指定再改。</t>
         </is>
       </c>
       <c r="L12" s="28" t="n">
@@ -2078,7 +2043,7 @@
       </c>
       <c r="C13" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
@@ -2088,7 +2053,7 @@
       </c>
       <c r="E13" s="29" t="inlineStr">
         <is>
-          <t>三片断厂家方案与原方案查漏补缺，合并为一套改造方案。</t>
+          <t>三片段厂家方案与原方案合并为一套改造方案。</t>
         </is>
       </c>
       <c r="F13" s="29" t="inlineStr">
@@ -2098,7 +2063,7 @@
       </c>
       <c r="G13" s="27" t="inlineStr">
         <is>
-          <t>志恒</t>
+          <t>王志恒</t>
         </is>
       </c>
       <c r="H13" s="28" t="n">
@@ -2116,7 +2081,7 @@
       </c>
       <c r="K13" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会明确：三片断方案合并后才算整套改造方案形成。</t>
+          <t>2026-09-21：IEPE 由王志恒、张国睿整体负责。</t>
         </is>
       </c>
       <c r="L13" s="28" t="n">
@@ -2143,7 +2108,7 @@
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D14" s="30" t="inlineStr">
@@ -2153,7 +2118,7 @@
       </c>
       <c r="E14" s="29" t="inlineStr">
         <is>
-          <t>列出配液「利旧改造 vs 推倒重建」对比，单独报领导。</t>
+          <t>配液利旧还是推倒，方案列出后报领导。</t>
         </is>
       </c>
       <c r="F14" s="29" t="inlineStr">
@@ -2163,7 +2128,7 @@
       </c>
       <c r="G14" s="27" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="H14" s="28" t="n"/>
@@ -2179,7 +2144,7 @@
       </c>
       <c r="K14" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：会上明确未决，方案列出后单独汇报。</t>
+          <t>2026-09-21：会上明确未决。</t>
         </is>
       </c>
       <c r="L14" s="28" t="n">
@@ -2206,7 +2171,7 @@
       </c>
       <c r="C15" s="29" t="inlineStr">
         <is>
-          <t>方哥/王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
@@ -2216,12 +2181,12 @@
       </c>
       <c r="E15" s="29" t="inlineStr">
         <is>
-          <t>输出采购三类台账：已采买、询价中、未采购；此后每日更新到货进展。</t>
+          <t>交出 139788 项目采购总台账，三类写清：已下单采买、询价中、尚未采购。</t>
         </is>
       </c>
       <c r="F15" s="29" t="inlineStr">
         <is>
-          <t>物料可点名归入三类之一；每日有更新。</t>
+          <t>总台账可按三类点名到物料。</t>
         </is>
       </c>
       <c r="G15" s="27" t="inlineStr">
@@ -2244,7 +2209,7 @@
       </c>
       <c r="K15" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：部署会布置。田子才、冯毅配合；三人无论谁在场，每天向主持更新到货。</t>
+          <t>2026-09-21：总指挥指定宋金柱跟采购同事今天出总账。工程亦由宋金柱整体负责。</t>
         </is>
       </c>
       <c r="L15" s="28" t="n">
@@ -2261,66 +2226,66 @@
       </c>
     </row>
     <row r="16" ht="56" customHeight="1">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>A-20260921-12</t>
         </is>
       </c>
-      <c r="B16" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="C16" s="29" t="inlineStr">
-        <is>
-          <t>方哥</t>
-        </is>
-      </c>
-      <c r="D16" s="30" t="inlineStr">
+      <c r="B16" s="32" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>张俊峰</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
         <is>
           <t>采购到货</t>
         </is>
       </c>
-      <c r="E16" s="29" t="inlineStr">
-        <is>
-          <t>核实东富龙 600 搅拌罐采购订货状态。</t>
-        </is>
-      </c>
-      <c r="F16" s="29" t="inlineStr">
-        <is>
-          <t>订货状态写入台账。</t>
-        </is>
-      </c>
-      <c r="G16" s="27" t="inlineStr">
-        <is>
-          <t>宋金柱</t>
-        </is>
-      </c>
-      <c r="H16" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="I16" s="27" t="inlineStr">
-        <is>
-          <t>未开始</t>
-        </is>
-      </c>
-      <c r="J16" s="30" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="K16" s="29" t="inlineStr">
-        <is>
-          <t>2026-09-21：部署会指定为金柱今日重点之一。</t>
-        </is>
-      </c>
-      <c r="L16" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="M16" s="29" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>冯毅、田子才每日在群里上报采购与到货进展。</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>群里每日有进展，不空报。</t>
+        </is>
+      </c>
+      <c r="G16" s="31" t="inlineStr">
+        <is>
+          <t>冯毅</t>
+        </is>
+      </c>
+      <c r="H16" s="32" t="n">
+        <v>46286</v>
+      </c>
+      <c r="I16" s="31" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="J16" s="34" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K16" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-21：总指挥指定冯毅、田子才后续每日上报，不是冯毅+宋金柱双主责日报。</t>
+        </is>
+      </c>
+      <c r="L16" s="32" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M16" s="33" t="inlineStr">
         <is>
           <t>2026-09-21 部署会</t>
         </is>
       </c>
-      <c r="N16" s="30">
+      <c r="N16" s="34">
         <f>IF(OR(I16="已完成",I16="取消"),"—",IF(H16="",IF(I16="阻塞","逾期","—"),IF(H16&lt;TODAY(),"逾期",IF(H16=TODAY(),"今日到期","按期"))))</f>
         <v/>
       </c>
@@ -2336,7 +2301,7 @@
       </c>
       <c r="C17" s="29" t="inlineStr">
         <is>
-          <t>方哥</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D17" s="30" t="inlineStr">
@@ -2346,17 +2311,17 @@
       </c>
       <c r="E17" s="29" t="inlineStr">
         <is>
-          <t>湿氮气擦净、消毒、推至车间门口，再拆卸转移至 AFD（三合一）背后；中午前完成。</t>
+          <t>湿氮气擦净、消毒、中午前转移至 AFD（三合一）后侧。</t>
         </is>
       </c>
       <c r="F17" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21 13:00 客户进车间前就位并复确认擦洗。</t>
+          <t>13:00 客户进车间前就位。</t>
         </is>
       </c>
       <c r="G17" s="27" t="inlineStr">
         <is>
-          <t>宋金柱</t>
+          <t>郭泽鹏</t>
         </is>
       </c>
       <c r="H17" s="28" t="n">
@@ -2374,7 +2339,7 @@
       </c>
       <c r="K17" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：泽鹏进场后第一时间擦净推到物流通道，消完毒推到车间门口；其后金柱安排拆卸，转移到 AFD 背后。中午前完成。</t>
+          <t>2026-09-21：郭泽鹏运到门口；宋金柱安排拆卸转移。郭泽鹏 50% 精力在整改，今日跟王志恒和厂家走现场。</t>
         </is>
       </c>
       <c r="L17" s="28" t="n">
@@ -2401,7 +2366,7 @@
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D18" s="30" t="inlineStr">
@@ -2416,7 +2381,7 @@
       </c>
       <c r="F18" s="29" t="inlineStr">
         <is>
-          <t>分工与计划已对接主持侧。</t>
+          <t>分工与计划已对接总指挥侧。</t>
         </is>
       </c>
       <c r="G18" s="27" t="inlineStr">
@@ -2439,7 +2404,7 @@
       </c>
       <c r="K18" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：王总已电话沟通；会中明确后天到岗。QA 美佳后续与其交底。</t>
+          <t>2026-09-21：会中明确后天到岗。QA 等 DH 支持后再交底。</t>
         </is>
       </c>
       <c r="L18" s="28" t="n">
@@ -2456,66 +2421,66 @@
       </c>
     </row>
     <row r="19" ht="56" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="35" t="inlineStr">
         <is>
           <t>A-20260921-15</t>
         </is>
       </c>
-      <c r="B19" s="32" t="n">
-        <v>46286</v>
-      </c>
-      <c r="C19" s="33" t="inlineStr">
-        <is>
-          <t>美佳</t>
-        </is>
-      </c>
-      <c r="D19" s="34" t="inlineStr">
+      <c r="B19" s="36" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>刘美佳</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
         <is>
           <t>制备配液</t>
         </is>
       </c>
-      <c r="E19" s="33" t="inlineStr">
-        <is>
-          <t>向腾信压缩 D 区现有搅拌罐改口工期；达不成则把完不成节点提到中午沟通会。</t>
-        </is>
-      </c>
-      <c r="F19" s="33" t="inlineStr">
-        <is>
-          <t>新工期，或正式报出的冲突节点（洪杰 / 美佳 / 张豹可上会）。</t>
-        </is>
-      </c>
-      <c r="G19" s="31" t="inlineStr">
-        <is>
-          <t>美佳</t>
-        </is>
-      </c>
-      <c r="H19" s="32" t="n">
-        <v>46286</v>
-      </c>
-      <c r="I19" s="31" t="inlineStr">
+      <c r="E19" s="37" t="inlineStr">
+        <is>
+          <t>向腾信压缩 D 区现有搅拌罐改口工期；达不成则把完不成节点报到中午沟通会。</t>
+        </is>
+      </c>
+      <c r="F19" s="37" t="inlineStr">
+        <is>
+          <t>新工期，或正式报出的冲突节点。</t>
+        </is>
+      </c>
+      <c r="G19" s="35" t="inlineStr">
+        <is>
+          <t>刘美佳</t>
+        </is>
+      </c>
+      <c r="H19" s="36" t="n">
+        <v>46286</v>
+      </c>
+      <c r="I19" s="35" t="inlineStr">
         <is>
           <t>阻塞</t>
         </is>
       </c>
-      <c r="J19" s="34" t="inlineStr">
+      <c r="J19" s="38" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="K19" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-21：美佳反馈约 5 个罐、工期 20 天（15 日起改到下月 5 日），与 11/18 交付冲突；并判断 20 天也不一定做完。王总/方哥要求继续压，资源不够找郭宏杰。</t>
-        </is>
-      </c>
-      <c r="L19" s="32" t="n">
-        <v>46286</v>
-      </c>
-      <c r="M19" s="33" t="inlineStr">
+      <c r="K19" s="37" t="inlineStr">
+        <is>
+          <t>2026-09-21：约 5 台、工期 20 天，与 11/18 冲突。资源不够找郭宏杰。初稿误写诚信、徐瑞。</t>
+        </is>
+      </c>
+      <c r="L19" s="36" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M19" s="37" t="inlineStr">
         <is>
           <t>2026-09-21 部署会</t>
         </is>
       </c>
-      <c r="N19" s="34">
+      <c r="N19" s="38">
         <f>IF(OR(I19="已完成",I19="取消"),"—",IF(H19="",IF(I19="阻塞","逾期","—"),IF(H19&lt;TODAY(),"逾期",IF(H19=TODAY(),"今日到期","按期"))))</f>
         <v/>
       </c>
@@ -2531,7 +2496,7 @@
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>方哥</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D20" s="30" t="inlineStr">
@@ -2541,17 +2506,17 @@
       </c>
       <c r="E20" s="29" t="inlineStr">
         <is>
-          <t>先出既有采购清单，再把客户新加项与厂家新识别改造项补入。</t>
+          <t>总台账先出既有项，再补客户新加项和厂家新识别项。</t>
         </is>
       </c>
       <c r="F20" s="29" t="inlineStr">
         <is>
-          <t>新旧项可区分，不回头混在一起。</t>
+          <t>新旧项可区分。</t>
         </is>
       </c>
       <c r="G20" s="27" t="inlineStr">
         <is>
-          <t>美佳</t>
+          <t>宋金柱</t>
         </is>
       </c>
       <c r="H20" s="28" t="n">
@@ -2569,7 +2534,7 @@
       </c>
       <c r="K20" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：客户刚新加多项；厂家今日仍在梳理，梳理完往清单里补。自控阀门货期可能拖交付。</t>
+          <t>2026-09-21：与 A-11 联动。</t>
         </is>
       </c>
       <c r="L20" s="28" t="n">
@@ -2586,66 +2551,66 @@
       </c>
     </row>
     <row r="21" ht="56" customHeight="1">
-      <c r="A21" s="35" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>A-20260921-17</t>
         </is>
       </c>
-      <c r="B21" s="36" t="n">
-        <v>46286</v>
-      </c>
-      <c r="C21" s="37" t="inlineStr">
-        <is>
-          <t>王总</t>
-        </is>
-      </c>
-      <c r="D21" s="38" t="inlineStr">
+      <c r="B21" s="32" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>张俊峰</t>
+        </is>
+      </c>
+      <c r="D21" s="34" t="inlineStr">
         <is>
           <t>综合协调</t>
         </is>
       </c>
-      <c r="E21" s="37" t="inlineStr">
-        <is>
-          <t>组织每日 19:00 改造沟通会（含线上）。</t>
-        </is>
-      </c>
-      <c r="F21" s="37" t="inlineStr">
-        <is>
-          <t>会议召开，行动项有当日进展。</t>
-        </is>
-      </c>
-      <c r="G21" s="35" t="inlineStr">
-        <is>
-          <t>德鹏</t>
-        </is>
-      </c>
-      <c r="H21" s="36" t="n">
-        <v>46286</v>
-      </c>
-      <c r="I21" s="35" t="inlineStr">
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>每日 19:00 改造沟通会（可线上）；周一早晨约 30 分钟同步。</t>
+        </is>
+      </c>
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>会议召开，当日行动有进展。</t>
+        </is>
+      </c>
+      <c r="G21" s="31" t="inlineStr">
+        <is>
+          <t>张俊峰</t>
+        </is>
+      </c>
+      <c r="H21" s="32" t="n">
+        <v>46286</v>
+      </c>
+      <c r="I21" s="31" t="inlineStr">
         <is>
           <t>进行中</t>
         </is>
       </c>
-      <c r="J21" s="38" t="inlineStr">
+      <c r="J21" s="34" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="K21" s="37" t="inlineStr">
-        <is>
-          <t>2026-09-21：部署会确定每晚 19:00；可线上。另议周一晨会半小时，是否固定待确认。</t>
-        </is>
-      </c>
-      <c r="L21" s="36" t="n">
-        <v>46286</v>
-      </c>
-      <c r="M21" s="37" t="inlineStr">
+      <c r="K21" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-21：总指挥要求全员参加。初稿写「德鹏组织」未再核实，主责记总指挥。</t>
+        </is>
+      </c>
+      <c r="L21" s="32" t="n">
+        <v>46286</v>
+      </c>
+      <c r="M21" s="33" t="inlineStr">
         <is>
           <t>2026-09-21 部署会</t>
         </is>
       </c>
-      <c r="N21" s="38">
+      <c r="N21" s="34">
         <f>IF(OR(I21="已完成",I21="取消"),"—",IF(H21="",IF(I21="阻塞","逾期","—"),IF(H21&lt;TODAY(),"逾期",IF(H21=TODAY(),"今日到期","按期"))))</f>
         <v/>
       </c>
@@ -2661,7 +2626,7 @@
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>李方向</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D22" s="30" t="inlineStr">
@@ -2671,20 +2636,22 @@
       </c>
       <c r="E22" s="29" t="inlineStr">
         <is>
-          <t>为张东申请电脑。</t>
+          <t>郭泽鹏 50% 精力投入整改，今日跟王志恒和厂家完成车间勘察跟踪。</t>
         </is>
       </c>
       <c r="F22" s="29" t="inlineStr">
         <is>
-          <t>电脑到位。</t>
+          <t>现场有跟，不代替王志恒出清单。</t>
         </is>
       </c>
       <c r="G22" s="27" t="inlineStr">
         <is>
-          <t>李方向</t>
-        </is>
-      </c>
-      <c r="H22" s="28" t="n"/>
+          <t>郭泽鹏</t>
+        </is>
+      </c>
+      <c r="H22" s="28" t="n">
+        <v>46286</v>
+      </c>
       <c r="I22" s="27" t="inlineStr">
         <is>
           <t>未开始</t>
@@ -2692,12 +2659,12 @@
       </c>
       <c r="J22" s="30" t="inlineStr">
         <is>
-          <t>低</t>
+          <t>中</t>
         </is>
       </c>
       <c r="K22" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：会上确认张东无电脑，李方向答应申请。</t>
+          <t>2026-09-21：总指挥明确是配合和学习，不是三个片段总协调。</t>
         </is>
       </c>
       <c r="L22" s="28" t="n">
@@ -2724,7 +2691,7 @@
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
-          <t>李方向</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
@@ -2734,17 +2701,17 @@
       </c>
       <c r="E23" s="29" t="inlineStr">
         <is>
-          <t>在 demo 批次启动前完成设计，并报客户沟通敲定，避免边改边设计。</t>
+          <t>10 月中下旬前完成设计并报客户敲定，避免边改边设计。</t>
         </is>
       </c>
       <c r="F23" s="29" t="inlineStr">
         <is>
-          <t>客户确认方案；不耽误 10 月中下旬开工。</t>
+          <t>客户确认方案。</t>
         </is>
       </c>
       <c r="G23" s="27" t="inlineStr">
         <is>
-          <t>待指定（生产部 + IPE）</t>
+          <t>王志恒</t>
         </is>
       </c>
       <c r="H23" s="28" t="n">
@@ -2762,7 +2729,7 @@
       </c>
       <c r="K23" s="29" t="inlineStr">
         <is>
-          <t>2026-09-21：李方向强调设计须在 10 月中下旬前搞定。IPE 厂家与生产部整体负责，确认后报客户。</t>
+          <t>2026-09-21：IEPE 王志恒、张国睿整体负责。截止日期 10/20 为纪要推断，待核实。</t>
         </is>
       </c>
       <c r="L23" s="28" t="n">
@@ -3231,12 +3198,12 @@
       </c>
       <c r="B4" s="22" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C4" s="22" t="inlineStr">
         <is>
-          <t>牵头东富龙现场，按设备本体 / 管道 / 仪表 / 阀门 / 泵查漏补缺，更新制备配液与超滤改造须知。</t>
+          <t>打印改造事项清单；与东富龙技术员逐管路、逐设备过制备配液和超滤，缺项补进同一清单。</t>
         </is>
       </c>
       <c r="D4" s="22">
@@ -3248,7 +3215,7 @@
         <v/>
       </c>
       <c r="F4" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G4,'行动项总账'!$A:$A,0)),"志恒")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G4,'行动项总账'!$A:$A,0)),"王志恒")</f>
         <v/>
       </c>
       <c r="G4" s="42" t="inlineStr">
@@ -3263,12 +3230,12 @@
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>对接东富龙现场人员，完成上午车间勘察。</t>
+          <t>负责制备配液和制备工序整改；今日跟王志恒、东富龙走现场并跟踪本片段。</t>
         </is>
       </c>
       <c r="D5" s="20">
@@ -3280,7 +3247,7 @@
         <v/>
       </c>
       <c r="F5" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G5,'行动项总账'!$A:$A,0)),"李主任")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G5,'行动项总账'!$A:$A,0)),"皮轶杰")</f>
         <v/>
       </c>
       <c r="G5" s="45" t="inlineStr">
@@ -3295,12 +3262,12 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C6" s="22" t="inlineStr">
         <is>
-          <t>跟点超滤片断现场勘察并记录缺项。</t>
+          <t>负责超滤工序整改；今日跟王志恒、东富龙走现场并记录缺项。</t>
         </is>
       </c>
       <c r="D6" s="22">
@@ -3312,7 +3279,7 @@
         <v/>
       </c>
       <c r="F6" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G6,'行动项总账'!$A:$A,0)),"张东")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G6,'行动项总账'!$A:$A,0)),"张冬")</f>
         <v/>
       </c>
       <c r="G6" s="42" t="inlineStr">
@@ -3327,12 +3294,12 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>厂家技术配合结束后，梳理超滤 / 制备配液改造事项并提交下午会。</t>
+          <t>负责沉淀工序整改；13:00 跟王志恒、亚光过沉淀区域。</t>
         </is>
       </c>
       <c r="D7" s="20">
@@ -3344,7 +3311,7 @@
         <v/>
       </c>
       <c r="F7" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G7,'行动项总账'!$A:$A,0)),"志鹏")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G7,'行动项总账'!$A:$A,0)),"韩瑞衡")</f>
         <v/>
       </c>
       <c r="G7" s="45" t="inlineStr">
@@ -3359,12 +3326,12 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C8" s="22" t="inlineStr">
         <is>
-          <t>按沉淀 / 超滤 / 制备三片断，评估客户访问问题是否举一反三全覆盖，写入表单。</t>
+          <t>梳理客户来访全部问题，核三个片段涉及整改的内容是否都举一反三、都有整改要求。</t>
         </is>
       </c>
       <c r="D8" s="22">
@@ -3376,7 +3343,7 @@
         <v/>
       </c>
       <c r="F8" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G8,'行动项总账'!$A:$A,0)),"松涛")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G8,'行动项总账'!$A:$A,0)),"范兴涛")</f>
         <v/>
       </c>
       <c r="G8" s="42" t="inlineStr">
@@ -3391,12 +3358,12 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>王（IAP）</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>通知东富龙曹工 / 赵工上午到场勘察利旧，下午交出利旧与推倒两套方案对比。</t>
+          <t>对接东富龙，下午交出利旧与推倒重建两套方案的时间/事项对比。</t>
         </is>
       </c>
       <c r="D9" s="20">
@@ -3408,7 +3375,7 @@
         <v/>
       </c>
       <c r="F9" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G9,'行动项总账'!$A:$A,0)),"王（IAP，全名待补）")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G9,'行动项总账'!$A:$A,0)),"王志恒")</f>
         <v/>
       </c>
       <c r="G9" s="45" t="inlineStr">
@@ -3423,12 +3390,12 @@
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C10" s="22" t="inlineStr">
         <is>
-          <t>13:00 与亚光（菊工）合并昨天下午勘察事项与内部清单。</t>
+          <t>13:00 与亚光技术员梳理沉淀区域整改项，更新同一份改造清单。</t>
         </is>
       </c>
       <c r="D10" s="22">
@@ -3440,7 +3407,7 @@
         <v/>
       </c>
       <c r="F10" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G10,'行动项总账'!$A:$A,0)),"王总")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G10,'行动项总账'!$A:$A,0)),"王志恒")</f>
         <v/>
       </c>
       <c r="G10" s="42" t="inlineStr">
@@ -3455,7 +3422,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
@@ -3472,7 +3439,7 @@
         <v/>
       </c>
       <c r="F11" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G11,'行动项总账'!$A:$A,0)),"汉邦对接人（待补）")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G11,'行动项总账'!$A:$A,0)),"王志恒")</f>
         <v/>
       </c>
       <c r="G11" s="45" t="inlineStr">
@@ -3487,12 +3454,12 @@
       </c>
       <c r="B12" s="22" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
         <is>
-          <t>三片断厂家方案与原方案查漏补缺，合并为一套改造方案。</t>
+          <t>三片段厂家方案与原方案合并为一套改造方案。</t>
         </is>
       </c>
       <c r="D12" s="22">
@@ -3504,7 +3471,7 @@
         <v/>
       </c>
       <c r="F12" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G12,'行动项总账'!$A:$A,0)),"志恒")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G12,'行动项总账'!$A:$A,0)),"王志恒")</f>
         <v/>
       </c>
       <c r="G12" s="42" t="inlineStr">
@@ -3519,12 +3486,12 @@
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>列出配液「利旧改造 vs 推倒重建」对比，单独报领导。</t>
+          <t>配液利旧还是推倒，方案列出后报领导。</t>
         </is>
       </c>
       <c r="D13" s="20">
@@ -3536,7 +3503,7 @@
         <v/>
       </c>
       <c r="F13" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G13,'行动项总账'!$A:$A,0)),"王总")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G13,'行动项总账'!$A:$A,0)),"张俊峰")</f>
         <v/>
       </c>
       <c r="G13" s="45" t="inlineStr">
@@ -3551,12 +3518,12 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>方哥/王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C14" s="22" t="inlineStr">
         <is>
-          <t>输出采购三类台账：已采买、询价中、未采购；此后每日更新到货进展。</t>
+          <t>交出 139788 项目采购总台账，三类写清：已下单采买、询价中、尚未采购。</t>
         </is>
       </c>
       <c r="D14" s="22">
@@ -3583,12 +3550,12 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>方哥</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>核实东富龙 600 搅拌罐采购订货状态。</t>
+          <t>冯毅、田子才每日在群里上报采购与到货进展。</t>
         </is>
       </c>
       <c r="D15" s="20">
@@ -3600,7 +3567,7 @@
         <v/>
       </c>
       <c r="F15" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G15,'行动项总账'!$A:$A,0)),"宋金柱")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G15,'行动项总账'!$A:$A,0)),"冯毅")</f>
         <v/>
       </c>
       <c r="G15" s="45" t="inlineStr">
@@ -3615,12 +3582,12 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>方哥</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C16" s="22" t="inlineStr">
         <is>
-          <t>湿氮气擦净、消毒、推至车间门口，再拆卸转移至 AFD（三合一）背后；中午前完成。</t>
+          <t>湿氮气擦净、消毒、中午前转移至 AFD（三合一）后侧。</t>
         </is>
       </c>
       <c r="D16" s="22">
@@ -3632,7 +3599,7 @@
         <v/>
       </c>
       <c r="F16" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G16,'行动项总账'!$A:$A,0)),"宋金柱")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G16,'行动项总账'!$A:$A,0)),"郭泽鹏")</f>
         <v/>
       </c>
       <c r="G16" s="42" t="inlineStr">
@@ -3647,7 +3614,7 @@
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr">
@@ -3674,32 +3641,32 @@
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="32" t="n">
-        <v>46286</v>
-      </c>
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>美佳</t>
-        </is>
-      </c>
-      <c r="C18" s="33" t="inlineStr">
-        <is>
-          <t>向腾信压缩 D 区现有搅拌罐改口工期；达不成则把完不成节点提到中午沟通会。</t>
-        </is>
-      </c>
-      <c r="D18" s="33">
+      <c r="A18" s="36" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>刘美佳</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>向腾信压缩 D 区现有搅拌罐改口工期；达不成则把完不成节点报到中午沟通会。</t>
+        </is>
+      </c>
+      <c r="D18" s="37">
         <f>IFERROR(INDEX('行动项总账'!$K:$K,MATCH(G18,'行动项总账'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="E18" s="31">
+      <c r="E18" s="35">
         <f>IFERROR(IF(INDEX('行动项总账'!$I:$I,MATCH(G18,'行动项总账'!$A:$A,0))="已完成","YES",IF(INDEX('行动项总账'!$I:$I,MATCH(G18,'行动项总账'!$A:$A,0))="阻塞","BLOCKED","NO")),"NO")</f>
         <v/>
       </c>
       <c r="F18" s="47">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G18,'行动项总账'!$A:$A,0)),"美佳")</f>
-        <v/>
-      </c>
-      <c r="G18" s="31" t="inlineStr">
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G18,'行动项总账'!$A:$A,0)),"刘美佳")</f>
+        <v/>
+      </c>
+      <c r="G18" s="35" t="inlineStr">
         <is>
           <t>A-20260921-15</t>
         </is>
@@ -3711,12 +3678,12 @@
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>方哥</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C19" s="20" t="inlineStr">
         <is>
-          <t>先出既有采购清单，再把客户新加项与厂家新识别改造项补入。</t>
+          <t>总台账先出既有项，再补客户新加项和厂家新识别项。</t>
         </is>
       </c>
       <c r="D19" s="20">
@@ -3728,7 +3695,7 @@
         <v/>
       </c>
       <c r="F19" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G19,'行动项总账'!$A:$A,0)),"美佳")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G19,'行动项总账'!$A:$A,0)),"宋金柱")</f>
         <v/>
       </c>
       <c r="G19" s="45" t="inlineStr">
@@ -3743,12 +3710,12 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>王总</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C20" s="22" t="inlineStr">
         <is>
-          <t>组织每日 19:00 改造沟通会（含线上）。</t>
+          <t>每日 19:00 改造沟通会（可线上）；周一早晨约 30 分钟同步。</t>
         </is>
       </c>
       <c r="D20" s="22">
@@ -3760,7 +3727,7 @@
         <v/>
       </c>
       <c r="F20" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G20,'行动项总账'!$A:$A,0)),"德鹏")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G20,'行动项总账'!$A:$A,0)),"张俊峰")</f>
         <v/>
       </c>
       <c r="G20" s="42" t="inlineStr">
@@ -3775,12 +3742,12 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>李方向</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C21" s="20" t="inlineStr">
         <is>
-          <t>为张东申请电脑。</t>
+          <t>郭泽鹏 50% 精力投入整改，今日跟王志恒和厂家完成车间勘察跟踪。</t>
         </is>
       </c>
       <c r="D21" s="20">
@@ -3792,7 +3759,7 @@
         <v/>
       </c>
       <c r="F21" s="46">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G21,'行动项总账'!$A:$A,0)),"李方向")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G21,'行动项总账'!$A:$A,0)),"郭泽鹏")</f>
         <v/>
       </c>
       <c r="G21" s="45" t="inlineStr">
@@ -3807,12 +3774,12 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>李方向</t>
+          <t>张俊峰</t>
         </is>
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
-          <t>在 demo 批次启动前完成设计，并报客户沟通敲定，避免边改边设计。</t>
+          <t>10 月中下旬前完成设计并报客户敲定，避免边改边设计。</t>
         </is>
       </c>
       <c r="D22" s="22">
@@ -3824,7 +3791,7 @@
         <v/>
       </c>
       <c r="F22" s="43">
-        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G22,'行动项总账'!$A:$A,0)),"待指定（生产部 + IPE）")</f>
+        <f>IFERROR(INDEX('行动项总账'!$G:$G,MATCH(G22,'行动项总账'!$A:$A,0)),"王志恒")</f>
         <v/>
       </c>
       <c r="G22" s="42" t="inlineStr">

</xml_diff>